<commit_message>
Ajustar responsables y horas del avance FARO
</commit_message>
<xml_diff>
--- a/datos/FARO_Cronograma_2026-08-13.xlsx
+++ b/datos/FARO_Cronograma_2026-08-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R7efd9ceb94ed4e9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R29636ed68d0f4393"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="3" r:id="Rf04b9de7365e46a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico avance" sheetId="4" r:id="R1672182527354c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R954dae04f9c84198"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Reac3247f09a443f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="3" r:id="R832d9d72819244c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico avance" sheetId="4" r:id="Rc3cfd8020688496d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38,10 +38,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
     <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
+    <x:numFmt numFmtId="202" formatCode="0.0"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -85,7 +86,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -166,6 +167,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -494,28 +496,28 @@
       <x:c r="G2" t="str">
         <x:v>Aarón Mayorga, Luis Martínez</x:v>
       </x:c>
-      <x:c r="H2" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I2" t="n">
+      <x:c r="H2" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I2" s="32" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J2" t="n">
+      <x:c r="J2" s="32" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K2" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L2" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M2" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N2" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O2" t="n">
+      <x:c r="K2" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L2" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M2" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N2" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O2" s="32" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="P2" s="13" t="str">
@@ -544,28 +546,28 @@
       <x:c r="G3" t="str">
         <x:v>Luis Montero, Aarón Mayorga, Karol</x:v>
       </x:c>
-      <x:c r="H3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I3" t="n">
+      <x:c r="H3" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I3" s="32" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="J3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L3" t="n">
+      <x:c r="J3" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L3" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="M3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O3" t="n">
+      <x:c r="M3" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N3" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O3" s="32" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="P3" s="13" t="str">
@@ -594,28 +596,28 @@
       <x:c r="G4" t="str">
         <x:v>Karol, Jorge Jiménez, Luis Montero</x:v>
       </x:c>
-      <x:c r="H4" t="n">
+      <x:c r="H4" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="I4" t="n">
+      <x:c r="I4" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="J4" t="n">
+      <x:c r="J4" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L4" t="n">
+      <x:c r="K4" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L4" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="M4" t="n">
+      <x:c r="M4" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="N4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O4" t="n">
+      <x:c r="N4" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O4" s="32" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="P4" s="13" t="str">
@@ -644,28 +646,28 @@
       <x:c r="G5" t="str">
         <x:v>Aarón Mayorga</x:v>
       </x:c>
-      <x:c r="H5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I5" t="n">
+      <x:c r="H5" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="32" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="J5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O5" t="n">
+      <x:c r="J5" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L5" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M5" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N5" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O5" s="32" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="P5" s="13"/>
@@ -690,34 +692,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>Daniel Pulido</x:v>
-      </x:c>
-      <x:c r="H6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K6" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="L6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O6" t="n">
-        <x:v>9</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H6" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="32" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="J6" s="32" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K6" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L6" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M6" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N6" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O6" s="32" t="n">
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="P6" s="13" t="str">
-        <x:v>Arquitectura lógica alineada al contexto canónico y al monolito modular; pendiente cierre formal.</x:v>
+        <x:v>Arquitectura lógica alineada al contexto canónico y al monolito modular; pendiente cierre formal. Equipo del avance: Aarón Mayorga 0.9 h y Luis Martínez 0.9 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -742,28 +744,28 @@
       <x:c r="G7" t="str">
         <x:v>Daniel Pulido</x:v>
       </x:c>
-      <x:c r="H7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O7" t="n">
+      <x:c r="H7" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L7" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N7" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O7" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P7" s="13" t="str">
@@ -792,28 +794,28 @@
       <x:c r="G8" t="str">
         <x:v>Daniel Pulido</x:v>
       </x:c>
-      <x:c r="H8" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I8" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J8" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K8" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L8" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M8" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N8" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O8" t="n">
+      <x:c r="H8" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L8" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M8" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N8" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O8" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P8" s="13" t="str">
@@ -840,34 +842,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>Daniel Pulido</x:v>
-      </x:c>
-      <x:c r="H9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K9" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="L9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O9" t="n">
-        <x:v>6</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H9" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="32" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J9" s="32" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="K9" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L9" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M9" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N9" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O9" s="32" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P9" s="13" t="str">
-        <x:v>Arquitectura modular documentada y aplicada; pendiente cierre formal.</x:v>
+        <x:v>Arquitectura modular documentada y aplicada; pendiente cierre formal. Equipo del avance: Aarón Mayorga 0.5 h y Luis Martínez 0.5 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -890,34 +892,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>Daniel Pulido</x:v>
-      </x:c>
-      <x:c r="H10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="L10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O10" t="n">
-        <x:v>2</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H10" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="32" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="J10" s="32" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="K10" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L10" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M10" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O10" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="P10" s="13" t="str">
-        <x:v>BFF, passwordless externo, capacidades y alcance reforzados; pendiente revisión final.</x:v>
+        <x:v>BFF, passwordless externo, capacidades y alcance reforzados; pendiente revisión final. Equipo del avance: Aarón Mayorga 0.7 h y Luis Martínez 0.7 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -942,32 +944,32 @@
       <x:c r="G11" t="str">
         <x:v>Aarón Mayorga, Luis Martínez</x:v>
       </x:c>
-      <x:c r="H11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I11" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="J11" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K11" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="L11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O11" t="n">
-        <x:v>50</x:v>
+      <x:c r="H11" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" s="32" t="n">
+        <x:v>2.9</x:v>
+      </x:c>
+      <x:c r="J11" s="32" t="n">
+        <x:v>2.9</x:v>
+      </x:c>
+      <x:c r="K11" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L11" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N11" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O11" s="32" t="n">
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="P11" s="13" t="str">
-        <x:v>Modelo canónico de pre-registro, IAM y GTRS implementado; pendientes de waves posteriores.</x:v>
+        <x:v>Modelo canónico de pre-registro, IAM y GTRS implementado; pendientes de waves posteriores. Equipo del avance: Aarón Mayorga 2.9 h y Luis Martínez 2.9 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -990,34 +992,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>Daniel Pulido, Aarón Mayorga</x:v>
-      </x:c>
-      <x:c r="H12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K12" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="L12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O12" t="n">
-        <x:v>10</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H12" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="32" t="n">
+        <x:v>4.7</x:v>
+      </x:c>
+      <x:c r="J12" s="32" t="n">
+        <x:v>4.7</x:v>
+      </x:c>
+      <x:c r="K12" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L12" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N12" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O12" s="32" t="n">
+        <x:v>9.4</x:v>
       </x:c>
       <x:c r="P12" s="13" t="str">
-        <x:v>Contratos canónicos de pre-registro, invitaciones y GTRS implementados y documentados; quedan verticales posteriores.</x:v>
+        <x:v>Contratos canónicos de pre-registro, invitaciones y GTRS implementados y documentados; quedan verticales posteriores. Equipo del avance: Aarón Mayorga 4.7 h y Luis Martínez 4.7 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1042,28 +1044,28 @@
       <x:c r="G13" t="str">
         <x:v>Daniel Pulido</x:v>
       </x:c>
-      <x:c r="H13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K13" t="n">
+      <x:c r="H13" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K13" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O13" t="n">
+      <x:c r="L13" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O13" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P13" s="13" t="str">
@@ -1090,34 +1092,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>Jorge Jiménez</x:v>
-      </x:c>
-      <x:c r="H14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K14" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O14" t="n">
-        <x:v>1</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H14" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" s="32" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="J14" s="32" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="K14" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L14" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M14" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N14" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O14" s="32" t="n">
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="P14" s="13" t="str">
-        <x:v>Ambiente local documentado; la configuración definitiva de Microsoft Entra por ambiente sigue pendiente.</x:v>
+        <x:v>Ambiente local documentado; la configuración definitiva de Microsoft Entra por ambiente sigue pendiente. Equipo del avance: Aarón Mayorga 0.1 h y Luis Martínez 0.1 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1142,28 +1144,28 @@
       <x:c r="G15" t="str">
         <x:v>Daniel Pulido, Luis Montero</x:v>
       </x:c>
-      <x:c r="H15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K15" t="n">
+      <x:c r="H15" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J15" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K15" s="32" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="L15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O15" t="n">
+      <x:c r="L15" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M15" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N15" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O15" s="32" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="P15" s="13" t="str">
@@ -1190,34 +1192,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>Daniel Pulido</x:v>
-      </x:c>
-      <x:c r="H16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O16" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H16" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="32" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="J16" s="32" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="K16" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L16" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M16" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N16" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O16" s="32" t="n">
+        <x:v>1.6</x:v>
       </x:c>
       <x:c r="P16" s="13" t="str">
-        <x:v>Pruebas frontend, backend, esquema y concurrencia disponibles; pendiente completar validación por ambientes.</x:v>
+        <x:v>Pruebas frontend, backend, esquema y concurrencia disponibles; pendiente completar validación por ambientes. Equipo del avance: Aarón Mayorga 0.8 h y Luis Martínez 0.8 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1240,34 +1242,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>Daniel Pulido, Jorge Jiménez</x:v>
-      </x:c>
-      <x:c r="H17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O17" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H17" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="32" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="J17" s="32" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="K17" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L17" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M17" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N17" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O17" s="32" t="n">
+        <x:v>2.4</x:v>
       </x:c>
       <x:c r="P17" s="13" t="str">
-        <x:v>CI de frontend, backend, esquema Supabase y contexto configurado; pendiente validar despliegue integral.</x:v>
+        <x:v>CI de frontend, backend, esquema Supabase y contexto configurado; pendiente validar despliegue integral. Equipo del avance: Aarón Mayorga 1.2 h y Luis Martínez 1.2 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1292,32 +1294,32 @@
       <x:c r="G18" t="str">
         <x:v>Aarón Mayorga, Luis Martínez</x:v>
       </x:c>
-      <x:c r="H18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K18" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="L18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O18" t="n">
-        <x:v>10</x:v>
+      <x:c r="H18" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="32" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="J18" s="32" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="K18" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L18" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M18" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N18" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O18" s="32" t="n">
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="P18" s="13" t="str">
-        <x:v>Esquema canónico, llaves y restricciones de pre-registro/GTRS implementados; pendientes de waves posteriores.</x:v>
+        <x:v>Esquema canónico, llaves y restricciones de pre-registro/GTRS implementados; pendientes de waves posteriores. Equipo del avance: Aarón Mayorga 3.3 h y Luis Martínez 3.3 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1340,34 +1342,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>Daniel Pulido, Aarón Mayorga</x:v>
-      </x:c>
-      <x:c r="H19" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I19" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J19" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K19" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="L19" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M19" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N19" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O19" t="n">
-        <x:v>2</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H19" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="32" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="J19" s="32" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="K19" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L19" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M19" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N19" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O19" s="32" t="n">
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="P19" s="13" t="str">
-        <x:v>RPC y funciones de pre-registro, invitaciones, GTRS, idempotencia y alcance global implementadas.</x:v>
+        <x:v>RPC y funciones de pre-registro, invitaciones, GTRS, idempotencia y alcance global implementadas. Equipo del avance: Aarón Mayorga 3.3 h y Luis Martínez 3.3 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1390,34 +1392,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>Daniel Pulido, Luis Montero, Jorge Jiménez</x:v>
-      </x:c>
-      <x:c r="H20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O20" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H20" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="32" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="J20" s="32" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="K20" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L20" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M20" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N20" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O20" s="32" t="n">
+        <x:v>7</x:v>
       </x:c>
       <x:c r="P20" s="13" t="str">
-        <x:v>Automatizaciones y auditoría transaccional implementadas en flujos Core; cobertura de módulos posteriores pendiente.</x:v>
+        <x:v>Automatizaciones y auditoría transaccional implementadas en flujos Core; cobertura de módulos posteriores pendiente. Equipo del avance: Aarón Mayorga 3.5 h y Luis Martínez 3.5 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1440,34 +1442,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G21" t="str">
-        <x:v>Daniel Pulido, Aarón Mayorga</x:v>
-      </x:c>
-      <x:c r="H21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I21" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="J21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O21" t="n">
-        <x:v>7</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H21" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" s="32" t="n">
+        <x:v>2.6</x:v>
+      </x:c>
+      <x:c r="J21" s="32" t="n">
+        <x:v>2.6</x:v>
+      </x:c>
+      <x:c r="K21" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L21" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M21" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N21" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O21" s="32" t="n">
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="P21" s="13" t="str">
-        <x:v>RBAC, capacidades y alcance por firma/global endurecidos; aprovisionamiento Microsoft y configuración avanzada pendientes.</x:v>
+        <x:v>RBAC, capacidades y alcance por firma/global endurecidos; aprovisionamiento Microsoft y configuración avanzada pendientes. Equipo del avance: Aarón Mayorga 2.6 h y Luis Martínez 2.6 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1490,34 +1492,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>Aarón Mayorga, Luis Montero, Luis Martínez, Jorge Jiménez</x:v>
-      </x:c>
-      <x:c r="H22" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I22" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J22" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K22" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L22" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M22" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N22" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O22" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H22" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" s="32" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J22" s="32" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="K22" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L22" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M22" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N22" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O22" s="32" t="n">
+        <x:v>38</x:v>
       </x:c>
       <x:c r="P22" s="13" t="str">
-        <x:v>Pre-registro full-stack integrado en Administrativo: bandeja, creación, invitaciones, aceptación passwordless, auditoría e idempotencia. Pendientes clientes/tenants y aprovisionamiento Microsoft.</x:v>
+        <x:v>Pre-registro full-stack integrado en Administrativo: bandeja, creación, invitaciones, aceptación passwordless, auditoría e idempotencia. Pendientes clientes/tenants y aprovisionamiento Microsoft. Equipo del avance: Aarón Mayorga 19.0 h y Luis Martínez 19.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1540,34 +1542,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>Luis Montero, Aarón Mayorga</x:v>
-      </x:c>
-      <x:c r="H23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I23" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="J23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O23" t="n">
-        <x:v>70</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H23" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="32" t="n">
+        <x:v>24.1</x:v>
+      </x:c>
+      <x:c r="J23" s="32" t="n">
+        <x:v>24.1</x:v>
+      </x:c>
+      <x:c r="K23" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L23" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M23" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N23" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O23" s="32" t="n">
+        <x:v>48.2</x:v>
       </x:c>
       <x:c r="P23" s="13" t="str">
-        <x:v>Backend GTRS cerrado para 8 secciones, lectura, ETag y submit atómico; el frontend /formulario-gtrs-v2 aún usa definición y solicitud mock.</x:v>
+        <x:v>Backend GTRS cerrado para 8 secciones, lectura, ETag y submit atómico; el frontend /formulario-gtrs-v2 aún usa definición y solicitud mock. Equipo del avance: Aarón Mayorga 24.1 h y Luis Martínez 24.1 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1590,34 +1592,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>Aarón Mayorga, Luis Montero, Luis Martínez</x:v>
-      </x:c>
-      <x:c r="H24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O24" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H24" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="32" t="n">
+        <x:v>16.6</x:v>
+      </x:c>
+      <x:c r="J24" s="32" t="n">
+        <x:v>16.6</x:v>
+      </x:c>
+      <x:c r="K24" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M24" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N24" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O24" s="32" t="n">
+        <x:v>33.2</x:v>
       </x:c>
       <x:c r="P24" s="13" t="str">
-        <x:v>State machine, autorización y contratos de revisión presentes; integración funcional completa de revisión/UI pendiente.</x:v>
+        <x:v>State machine, autorización y contratos de revisión presentes; integración funcional completa de revisión/UI pendiente. Equipo del avance: Aarón Mayorga 16.6 h y Luis Martínez 16.6 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1640,34 +1642,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>Luis Martínez, Aarón Mayorga, Luis Montero</x:v>
-      </x:c>
-      <x:c r="H25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O25" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H25" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I25" s="32" t="n">
+        <x:v>27.6</x:v>
+      </x:c>
+      <x:c r="J25" s="32" t="n">
+        <x:v>27.6</x:v>
+      </x:c>
+      <x:c r="K25" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L25" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M25" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N25" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O25" s="32" t="n">
+        <x:v>55.2</x:v>
       </x:c>
       <x:c r="P25" s="13" t="str">
-        <x:v>Invitación, aceptación passwordless, Magic Link y acceso externo multiempresa implementados; captura GTRS vertical pendiente.</x:v>
+        <x:v>Invitación, aceptación passwordless, Magic Link y acceso externo multiempresa implementados; captura GTRS vertical pendiente. Equipo del avance: Aarón Mayorga 27.6 h y Luis Martínez 27.6 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1690,34 +1692,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>Luis Martínez, Aarón Mayorga, Luis Montero</x:v>
-      </x:c>
-      <x:c r="H26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O26" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H26" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I26" s="32" t="n">
+        <x:v>7.8</x:v>
+      </x:c>
+      <x:c r="J26" s="32" t="n">
+        <x:v>7.8</x:v>
+      </x:c>
+      <x:c r="K26" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M26" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N26" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O26" s="32" t="n">
+        <x:v>15.6</x:v>
       </x:c>
       <x:c r="P26" s="13" t="str">
-        <x:v>Pre-registro interno, guards, permisos y gestión de usuarios integrados; otros workspaces conservan mocks/prototipos.</x:v>
+        <x:v>Pre-registro interno, guards, permisos y gestión de usuarios integrados; otros workspaces conservan mocks/prototipos. Equipo del avance: Aarón Mayorga 7.8 h y Luis Martínez 7.8 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1742,28 +1744,28 @@
       <x:c r="G27" t="str">
         <x:v>Luis Montero, Aarón Mayorga, Luis Martínez</x:v>
       </x:c>
-      <x:c r="H27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O27" t="n">
+      <x:c r="H27" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I27" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J27" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K27" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L27" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M27" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N27" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O27" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P27" s="13" t="str">
@@ -1792,28 +1794,28 @@
       <x:c r="G28" t="str">
         <x:v>Aarón Mayorga, Luis Montero, Luis Martínez</x:v>
       </x:c>
-      <x:c r="H28" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I28" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J28" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K28" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L28" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M28" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N28" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O28" t="n">
+      <x:c r="H28" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I28" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K28" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M28" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N28" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O28" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P28" s="13" t="str">
@@ -1840,34 +1842,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G29" t="str">
-        <x:v>Luis Montero, Aarón Mayorga, Luis Martínez, Jorge Jiménez</x:v>
-      </x:c>
-      <x:c r="H29" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I29" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J29" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K29" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L29" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M29" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N29" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O29" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H29" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="32" t="n">
+        <x:v>5.9</x:v>
+      </x:c>
+      <x:c r="J29" s="32" t="n">
+        <x:v>5.9</x:v>
+      </x:c>
+      <x:c r="K29" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M29" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N29" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O29" s="32" t="n">
+        <x:v>11.8</x:v>
       </x:c>
       <x:c r="P29" s="13" t="str">
-        <x:v>Contexto canónico, handoffs, decisiones, autenticación, despliegue y runbooks actualizados al 10/08.</x:v>
+        <x:v>Contexto canónico, handoffs, decisiones, autenticación, despliegue y runbooks actualizados al 10/08. Equipo del avance: Aarón Mayorga 5.9 h y Luis Martínez 5.9 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1890,34 +1892,34 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="G30" t="str">
-        <x:v>Karol, Daniel Pulido, Luis Montero, Jorge Jiménez</x:v>
-      </x:c>
-      <x:c r="H30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O30" t="n">
-        <x:v>0</x:v>
+        <x:v>Aarón Mayorga, Luis Martínez</x:v>
+      </x:c>
+      <x:c r="H30" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="32" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="J30" s="32" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="K30" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N30" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O30" s="32" t="n">
+        <x:v>9</x:v>
       </x:c>
       <x:c r="P30" s="13" t="str">
-        <x:v>Cobertura automatizada amplia en frontend, API, Application, SQL y concurrencia; UAT aún no iniciado.</x:v>
+        <x:v>Cobertura automatizada amplia en frontend, API, Application, SQL y concurrencia; UAT aún no iniciado. Equipo del avance: Aarón Mayorga 4.5 h y Luis Martínez 4.5 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1942,28 +1944,28 @@
       <x:c r="G31" t="str">
         <x:v>Karol, Daniel Pulido, Luis Montero, Jorge Jiménez</x:v>
       </x:c>
-      <x:c r="H31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O31" t="n">
+      <x:c r="H31" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J31" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K31" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L31" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M31" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N31" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O31" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P31" s="13" t="str">
@@ -1992,28 +1994,28 @@
       <x:c r="G32" t="str">
         <x:v>Daniel Pulido, Aarón Mayorga, Luis Montero</x:v>
       </x:c>
-      <x:c r="H32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O32" t="n">
+      <x:c r="H32" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K32" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M32" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N32" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O32" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P32" s="13" t="str">
@@ -2042,28 +2044,28 @@
       <x:c r="G33" t="str">
         <x:v>Karol, Daniel Pulido, Luis Montero, Jorge Jiménez</x:v>
       </x:c>
-      <x:c r="H33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O33" t="n">
+      <x:c r="H33" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I33" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K33" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M33" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N33" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O33" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P33" s="13" t="str">
@@ -2092,28 +2094,28 @@
       <x:c r="G34" t="str">
         <x:v>Kenneth, Daniel Pulido, Luis Montero, Jorge Jiménez</x:v>
       </x:c>
-      <x:c r="H34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O34" t="n">
+      <x:c r="H34" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K34" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N34" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O34" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P34" s="13" t="str">
@@ -2142,28 +2144,28 @@
       <x:c r="G35" t="str">
         <x:v>Daniel Pulido, Luis Montero</x:v>
       </x:c>
-      <x:c r="H35" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I35" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J35" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K35" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L35" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M35" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N35" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O35" t="n">
+      <x:c r="H35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N35" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O35" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P35" s="13" t="str">
@@ -2192,28 +2194,28 @@
       <x:c r="G36" t="str">
         <x:v>Daniel Pulido, Luis Montero, Kenneth</x:v>
       </x:c>
-      <x:c r="H36" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I36" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J36" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K36" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L36" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M36" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N36" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O36" t="n">
+      <x:c r="H36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N36" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O36" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P36" s="13" t="str">
@@ -2242,28 +2244,28 @@
       <x:c r="G37" t="str">
         <x:v>Luis Montero, Aarón Mayorga, Kenneth</x:v>
       </x:c>
-      <x:c r="H37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O37" t="n">
+      <x:c r="H37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N37" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O37" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P37" s="13" t="str">
@@ -2292,28 +2294,28 @@
       <x:c r="G38" t="str">
         <x:v>Luis Montero, Aarón Mayorga, Karol</x:v>
       </x:c>
-      <x:c r="H38" t="n">
+      <x:c r="H38" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I38" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J38" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K38" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L38" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M38" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N38" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O38" t="n">
+      <x:c r="I38" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J38" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K38" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L38" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M38" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N38" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O38" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="P38" s="13" t="str">
@@ -2342,28 +2344,28 @@
       <x:c r="G39" t="str">
         <x:v>Karol, Kenneth</x:v>
       </x:c>
-      <x:c r="H39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O39" t="n">
+      <x:c r="H39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N39" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O39" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P39" s="13" t="str">
@@ -2392,28 +2394,28 @@
       <x:c r="G40" t="str">
         <x:v>Aarón Mayorga, Luis Montero</x:v>
       </x:c>
-      <x:c r="H40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O40" t="n">
+      <x:c r="H40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N40" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O40" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P40" s="13" t="str">
@@ -2442,28 +2444,28 @@
       <x:c r="G41" t="str">
         <x:v>Karol, Luis Montero</x:v>
       </x:c>
-      <x:c r="H41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O41" t="n">
+      <x:c r="H41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N41" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O41" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P41" s="13" t="str">
@@ -2492,28 +2494,28 @@
       <x:c r="G42" t="str">
         <x:v>Luis Montero, Aarón Mayorga</x:v>
       </x:c>
-      <x:c r="H42" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I42" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J42" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K42" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L42" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M42" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N42" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O42" t="n">
+      <x:c r="H42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N42" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O42" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P42" s="13" t="str">
@@ -2542,28 +2544,28 @@
       <x:c r="G43" t="str">
         <x:v>Aarón Mayorga, Luis Montero</x:v>
       </x:c>
-      <x:c r="H43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O43" t="n">
+      <x:c r="H43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N43" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O43" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P43" s="13" t="str">
@@ -2592,28 +2594,28 @@
       <x:c r="G44" t="str">
         <x:v>Karol, Aarón Mayorga</x:v>
       </x:c>
-      <x:c r="H44" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I44" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J44" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K44" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L44" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M44" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N44" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O44" t="n">
+      <x:c r="H44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N44" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O44" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P44" s="13" t="str">
@@ -2642,28 +2644,28 @@
       <x:c r="G45" t="str">
         <x:v>Luis Montero, Aarón Mayorga</x:v>
       </x:c>
-      <x:c r="H45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O45" t="n">
+      <x:c r="H45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N45" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O45" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P45" s="13" t="str">
@@ -2716,13 +2718,13 @@
       <x:c r="C2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D2" t="n">
+      <x:c r="D2" s="32" t="n">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="E2" t="n">
+      <x:c r="E2" s="32" t="n">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="F2" t="n">
+      <x:c r="F2" s="32" t="n">
         <x:v>100</x:v>
       </x:c>
     </x:row>
@@ -2736,13 +2738,13 @@
       <x:c r="C3" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D3" t="n">
+      <x:c r="D3" s="32" t="n">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="E3" t="n">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="F3" t="n">
+      <x:c r="E3" s="32" t="n">
+        <x:v>41.6</x:v>
+      </x:c>
+      <x:c r="F3" s="32" t="n">
         <x:v>92.8</x:v>
       </x:c>
     </x:row>
@@ -2756,13 +2758,13 @@
       <x:c r="C4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D4" t="n">
+      <x:c r="D4" s="32" t="n">
         <x:v>781</x:v>
       </x:c>
-      <x:c r="E4" t="n">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="F4" t="n">
+      <x:c r="E4" s="32" t="n">
+        <x:v>227.4</x:v>
+      </x:c>
+      <x:c r="F4" s="32" t="n">
         <x:v>49.1</x:v>
       </x:c>
     </x:row>
@@ -2776,13 +2778,13 @@
       <x:c r="C5" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D5" t="n">
+      <x:c r="D5" s="32" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="E5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" t="n">
+      <x:c r="E5" s="32" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F5" s="32" t="n">
         <x:v>17.8</x:v>
       </x:c>
     </x:row>
@@ -2796,13 +2798,13 @@
       <x:c r="C6" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D6" t="n">
+      <x:c r="D6" s="32" t="n">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="E6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F6" t="n">
+      <x:c r="E6" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2816,13 +2818,13 @@
       <x:c r="C7" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D7" t="n">
+      <x:c r="D7" s="32" t="n">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="E7" t="n">
+      <x:c r="E7" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F7" t="n">
+      <x:c r="F7" s="32" t="n">
         <x:v>2.3</x:v>
       </x:c>
     </x:row>
@@ -2868,10 +2870,10 @@
       <x:c r="C2" t="str">
         <x:v>50%</x:v>
       </x:c>
-      <x:c r="D2">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="E2">
+      <x:c r="D2" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E2" s="32" t="n">
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -2885,11 +2887,11 @@
       <x:c r="C3" t="str">
         <x:v>75%</x:v>
       </x:c>
-      <x:c r="D3">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E3">
-        <x:v>145</x:v>
+      <x:c r="D3" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E3" s="32" t="n">
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2902,11 +2904,11 @@
       <x:c r="C4" t="str">
         <x:v>45%</x:v>
       </x:c>
-      <x:c r="D4">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E4">
-        <x:v>32</x:v>
+      <x:c r="D4" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E4" s="32" t="n">
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2919,11 +2921,11 @@
       <x:c r="C5" t="str">
         <x:v>30%</x:v>
       </x:c>
-      <x:c r="D5">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E5">
-        <x:v>41</x:v>
+      <x:c r="D5" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E5" s="32" t="n">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2936,10 +2938,10 @@
       <x:c r="C6" t="str">
         <x:v>30%</x:v>
       </x:c>
-      <x:c r="D6">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E6">
+      <x:c r="D6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E6" s="32" t="n">
         <x:v>9</x:v>
       </x:c>
     </x:row>
@@ -2953,10 +2955,10 @@
       <x:c r="C7" t="str">
         <x:v>40%</x:v>
       </x:c>
-      <x:c r="D7">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E7">
+      <x:c r="D7" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E7" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -2970,10 +2972,10 @@
       <x:c r="C8" t="str">
         <x:v>10%</x:v>
       </x:c>
-      <x:c r="D8">
+      <x:c r="D8" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E8">
+      <x:c r="E8" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3069,7 +3071,7 @@
         <x:v>Primer corte validado contra código ejecutable, migraciones, endpoints, pruebas y configuración funcional. Medición operativa ponderada por horas planificadas.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="58" customHeight="1">
+    <x:row r="3" ht="110" customHeight="1">
       <x:c r="A3" s="27" t="n">
         <x:v>46247.75</x:v>
       </x:c>
@@ -3101,13 +3103,13 @@
         <x:v>fdbea06</x:v>
       </x:c>
       <x:c r="K3" s="31" t="str">
-        <x:v>Corte validado sobre FARO main@fdbea06. Pre-registro full-stack integrado dentro de Administrativo: creación, bandeja, invitación/reenvío/revocación, aceptación passwordless, auditoría, idempotencia y alcance global Riesgo/Admin. También se reconoce el cierre backend GTRS de 8 secciones con ETag y gate de completitud. Pendientes principales: integración vertical del frontend GTRS, aprovisionamiento Microsoft/Entra y UAT.</x:v>
+        <x:v>Corte validado sobre FARO main@fdbea06. Pre-registro full-stack integrado dentro de Administrativo: creación, bandeja, invitación/reenvío/revocación, aceptación passwordless, auditoría, idempotencia y alcance global Riesgo/Admin. También se reconoce el cierre backend GTRS de 8 secciones con ETag y gate de completitud. Pendientes principales: integración vertical del frontend GTRS, aprovisionamiento Microsoft/Entra y UAT. Horas del avance redistribuidas: 260.0 h totales, 130.0 h Aarón Mayorga y 130.0 h Luis Martínez; sin participación de Daniel Pulido, Luis Montero, Karol ni Jorge Jiménez en las tareas que avanzaron.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb12621b442744c88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0f84c146ade4c8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Contabilizar horas omitidas del corte FARO
</commit_message>
<xml_diff>
--- a/datos/FARO_Cronograma_2026-08-13.xlsx
+++ b/datos/FARO_Cronograma_2026-08-13.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R954dae04f9c84198"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Reac3247f09a443f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="3" r:id="R832d9d72819244c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico avance" sheetId="4" r:id="Rc3cfd8020688496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R6a0e8624d33b43b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Rce2e86b2a45644b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="3" r:id="Rfdf76408db084c8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico avance" sheetId="4" r:id="Rd3802cc8b72e442f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidencia horas" sheetId="5" r:id="R0763a54769af43f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44,7 +45,7 @@
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
     <x:numFmt numFmtId="202" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="2">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -56,8 +57,31 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF4F2D7F"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF2D2D2D"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="12"/>
+      <x:color rgb="FF7A3E00"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF1F6E8C"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -74,19 +98,54 @@
         <x:fgColor rgb="FFF2FAE2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4F2D7F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3EFF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2FAE2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F6E8C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5F6F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
         <x:color rgb="FFD5E3B7"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF9BD732"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -168,6 +227,51 @@
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -670,7 +774,7 @@
       <x:c r="O5" s="32" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="P5" s="13"/>
+      <x:c r="P5" s="13" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="n">
@@ -701,10 +805,10 @@
         <x:v>0.9</x:v>
       </x:c>
       <x:c r="J6" s="32" t="n">
-        <x:v>0.9</x:v>
+        <x:v>1.9</x:v>
       </x:c>
       <x:c r="K6" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="L6" s="32" t="n">
         <x:v>0</x:v>
@@ -716,10 +820,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O6" s="32" t="n">
-        <x:v>1.8</x:v>
+        <x:v>11.8</x:v>
       </x:c>
       <x:c r="P6" s="13" t="str">
-        <x:v>Arquitectura lógica alineada al contexto canónico y al monolito modular; pendiente cierre formal. Equipo del avance: Aarón Mayorga 0.9 h y Luis Martínez 0.9 h.</x:v>
+        <x:v>Arquitectura lógica alineada al contexto canónico y al monolito modular; pendiente cierre formal. Equipo del avance: Aarón Mayorga 0.9 h y Luis Martínez 0.9 h. Corte 14/07–04/08 (GitHub): Aarón 0.0 h; Luis Martínez 1.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -848,13 +952,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I9" s="32" t="n">
-        <x:v>0.5</x:v>
+        <x:v>3.5</x:v>
       </x:c>
       <x:c r="J9" s="32" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="K9" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L9" s="32" t="n">
         <x:v>0</x:v>
@@ -866,10 +970,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O9" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="P9" s="13" t="str">
-        <x:v>Arquitectura modular documentada y aplicada; pendiente cierre formal. Equipo del avance: Aarón Mayorga 0.5 h y Luis Martínez 0.5 h.</x:v>
+        <x:v>Arquitectura modular documentada y aplicada; pendiente cierre formal. Equipo del avance: Aarón Mayorga 0.5 h y Luis Martínez 0.5 h. Corte 14/07–04/08 (GitHub): Aarón 3.0 h; Luis Martínez 1.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -898,13 +1002,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="32" t="n">
-        <x:v>0.7</x:v>
+        <x:v>3.7</x:v>
       </x:c>
       <x:c r="J10" s="32" t="n">
-        <x:v>0.7</x:v>
+        <x:v>2.7</x:v>
       </x:c>
       <x:c r="K10" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L10" s="32" t="n">
         <x:v>0</x:v>
@@ -916,10 +1020,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O10" s="32" t="n">
-        <x:v>1.4</x:v>
+        <x:v>8.4</x:v>
       </x:c>
       <x:c r="P10" s="13" t="str">
-        <x:v>BFF, passwordless externo, capacidades y alcance reforzados; pendiente revisión final. Equipo del avance: Aarón Mayorga 0.7 h y Luis Martínez 0.7 h.</x:v>
+        <x:v>BFF, passwordless externo, capacidades y alcance reforzados; pendiente revisión final. Equipo del avance: Aarón Mayorga 0.7 h y Luis Martínez 0.7 h. Corte 14/07–04/08 (GitHub): Aarón 3.0 h; Luis Martínez 2.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -948,13 +1052,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="32" t="n">
-        <x:v>2.9</x:v>
+        <x:v>22.9</x:v>
       </x:c>
       <x:c r="J11" s="32" t="n">
-        <x:v>2.9</x:v>
+        <x:v>22.9</x:v>
       </x:c>
       <x:c r="K11" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="L11" s="32" t="n">
         <x:v>0</x:v>
@@ -966,7 +1070,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O11" s="32" t="n">
-        <x:v>5.8</x:v>
+        <x:v>55.8</x:v>
       </x:c>
       <x:c r="P11" s="13" t="str">
         <x:v>Modelo canónico de pre-registro, IAM y GTRS implementado; pendientes de waves posteriores. Equipo del avance: Aarón Mayorga 2.9 h y Luis Martínez 2.9 h.</x:v>
@@ -998,13 +1102,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I12" s="32" t="n">
-        <x:v>4.7</x:v>
+        <x:v>6.7</x:v>
       </x:c>
       <x:c r="J12" s="32" t="n">
-        <x:v>4.7</x:v>
+        <x:v>9.7</x:v>
       </x:c>
       <x:c r="K12" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="L12" s="32" t="n">
         <x:v>0</x:v>
@@ -1016,10 +1120,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O12" s="32" t="n">
-        <x:v>9.4</x:v>
+        <x:v>26.4</x:v>
       </x:c>
       <x:c r="P12" s="13" t="str">
-        <x:v>Contratos canónicos de pre-registro, invitaciones y GTRS implementados y documentados; quedan verticales posteriores. Equipo del avance: Aarón Mayorga 4.7 h y Luis Martínez 4.7 h.</x:v>
+        <x:v>Contratos canónicos de pre-registro, invitaciones y GTRS implementados y documentados; quedan verticales posteriores. Equipo del avance: Aarón Mayorga 4.7 h y Luis Martínez 4.7 h. Corte 14/07–04/08 (GitHub): Aarón 2.0 h; Luis Martínez 5.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1048,10 +1152,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I13" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J13" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K13" s="32" t="n">
         <x:v>4</x:v>
@@ -1066,10 +1170,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O13" s="32" t="n">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="P13" s="13" t="str">
-        <x:v> </x:v>
+        <x:v>Corte 14/07–04/08 (GitHub): Aarón 2.0 h; Luis Martínez 1.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1098,13 +1202,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I14" s="32" t="n">
-        <x:v>0.1</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="J14" s="32" t="n">
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="K14" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L14" s="32" t="n">
         <x:v>0</x:v>
@@ -1116,10 +1220,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O14" s="32" t="n">
-        <x:v>0.2</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="P14" s="13" t="str">
-        <x:v>Ambiente local documentado; la configuración definitiva de Microsoft Entra por ambiente sigue pendiente. Equipo del avance: Aarón Mayorga 0.1 h y Luis Martínez 0.1 h.</x:v>
+        <x:v>Ambiente local documentado; la configuración definitiva de Microsoft Entra por ambiente sigue pendiente. Equipo del avance: Aarón Mayorga 0.1 h y Luis Martínez 0.1 h. Corte 14/07–04/08 (GitHub): Aarón 1.0 h; Luis Martínez 0.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1148,10 +1252,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I15" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J15" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K15" s="32" t="n">
         <x:v>8</x:v>
@@ -1166,10 +1270,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O15" s="32" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="P15" s="13" t="str">
-        <x:v> </x:v>
+        <x:v>Corte 14/07–04/08 (GitHub): Aarón 2.0 h; Luis Martínez 2.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1198,10 +1302,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I16" s="32" t="n">
-        <x:v>0.8</x:v>
+        <x:v>2.8</x:v>
       </x:c>
       <x:c r="J16" s="32" t="n">
-        <x:v>0.8</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="K16" s="32" t="n">
         <x:v>0</x:v>
@@ -1216,10 +1320,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O16" s="32" t="n">
-        <x:v>1.6</x:v>
+        <x:v>7.6</x:v>
       </x:c>
       <x:c r="P16" s="13" t="str">
-        <x:v>Pruebas frontend, backend, esquema y concurrencia disponibles; pendiente completar validación por ambientes. Equipo del avance: Aarón Mayorga 0.8 h y Luis Martínez 0.8 h.</x:v>
+        <x:v>Pruebas frontend, backend, esquema y concurrencia disponibles; pendiente completar validación por ambientes. Equipo del avance: Aarón Mayorga 0.8 h y Luis Martínez 0.8 h. Corte 14/07–04/08 (GitHub): Aarón 2.0 h; Luis Martínez 4.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1248,10 +1352,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I17" s="32" t="n">
-        <x:v>1.2</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="J17" s="32" t="n">
-        <x:v>1.2</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="K17" s="32" t="n">
         <x:v>0</x:v>
@@ -1266,10 +1370,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O17" s="32" t="n">
-        <x:v>2.4</x:v>
+        <x:v>8.4</x:v>
       </x:c>
       <x:c r="P17" s="13" t="str">
-        <x:v>CI de frontend, backend, esquema Supabase y contexto configurado; pendiente validar despliegue integral. Equipo del avance: Aarón Mayorga 1.2 h y Luis Martínez 1.2 h.</x:v>
+        <x:v>CI de frontend, backend, esquema Supabase y contexto configurado; pendiente validar despliegue integral. Equipo del avance: Aarón Mayorga 1.2 h y Luis Martínez 1.2 h. Corte 14/07–04/08 (GitHub): Aarón 3.0 h; Luis Martínez 3.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1298,13 +1402,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I18" s="32" t="n">
-        <x:v>3.3</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="J18" s="32" t="n">
-        <x:v>3.3</x:v>
+        <x:v>10.3</x:v>
       </x:c>
       <x:c r="K18" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="L18" s="32" t="n">
         <x:v>0</x:v>
@@ -1316,10 +1420,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O18" s="32" t="n">
-        <x:v>6.6</x:v>
+        <x:v>24.6</x:v>
       </x:c>
       <x:c r="P18" s="13" t="str">
-        <x:v>Esquema canónico, llaves y restricciones de pre-registro/GTRS implementados; pendientes de waves posteriores. Equipo del avance: Aarón Mayorga 3.3 h y Luis Martínez 3.3 h.</x:v>
+        <x:v>Esquema canónico, llaves y restricciones de pre-registro/GTRS implementados; pendientes de waves posteriores. Equipo del avance: Aarón Mayorga 3.3 h y Luis Martínez 3.3 h. Corte 14/07–04/08 (GitHub): Aarón 1.0 h; Luis Martínez 7.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1348,13 +1452,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="32" t="n">
-        <x:v>3.3</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="J19" s="32" t="n">
-        <x:v>3.3</x:v>
+        <x:v>8.3</x:v>
       </x:c>
       <x:c r="K19" s="32" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L19" s="32" t="n">
         <x:v>0</x:v>
@@ -1366,10 +1470,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O19" s="32" t="n">
-        <x:v>6.6</x:v>
+        <x:v>14.6</x:v>
       </x:c>
       <x:c r="P19" s="13" t="str">
-        <x:v>RPC y funciones de pre-registro, invitaciones, GTRS, idempotencia y alcance global implementadas. Equipo del avance: Aarón Mayorga 3.3 h y Luis Martínez 3.3 h.</x:v>
+        <x:v>RPC y funciones de pre-registro, invitaciones, GTRS, idempotencia y alcance global implementadas. Equipo del avance: Aarón Mayorga 3.3 h y Luis Martínez 3.3 h. Corte 14/07–04/08 (GitHub): Aarón 1.0 h; Luis Martínez 5.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1401,7 +1505,7 @@
         <x:v>3.5</x:v>
       </x:c>
       <x:c r="J20" s="32" t="n">
-        <x:v>3.5</x:v>
+        <x:v>7.5</x:v>
       </x:c>
       <x:c r="K20" s="32" t="n">
         <x:v>0</x:v>
@@ -1416,10 +1520,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O20" s="32" t="n">
-        <x:v>7</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="P20" s="13" t="str">
-        <x:v>Automatizaciones y auditoría transaccional implementadas en flujos Core; cobertura de módulos posteriores pendiente. Equipo del avance: Aarón Mayorga 3.5 h y Luis Martínez 3.5 h.</x:v>
+        <x:v>Automatizaciones y auditoría transaccional implementadas en flujos Core; cobertura de módulos posteriores pendiente. Equipo del avance: Aarón Mayorga 3.5 h y Luis Martínez 3.5 h. Corte 14/07–04/08 (GitHub): Aarón 0.0 h; Luis Martínez 4.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1448,10 +1552,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I21" s="32" t="n">
-        <x:v>2.6</x:v>
+        <x:v>12.6</x:v>
       </x:c>
       <x:c r="J21" s="32" t="n">
-        <x:v>2.6</x:v>
+        <x:v>8.6</x:v>
       </x:c>
       <x:c r="K21" s="32" t="n">
         <x:v>0</x:v>
@@ -1466,10 +1570,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O21" s="32" t="n">
-        <x:v>5.2</x:v>
+        <x:v>21.2</x:v>
       </x:c>
       <x:c r="P21" s="13" t="str">
-        <x:v>RBAC, capacidades y alcance por firma/global endurecidos; aprovisionamiento Microsoft y configuración avanzada pendientes. Equipo del avance: Aarón Mayorga 2.6 h y Luis Martínez 2.6 h.</x:v>
+        <x:v>RBAC, capacidades y alcance por firma/global endurecidos; aprovisionamiento Microsoft y configuración avanzada pendientes. Equipo del avance: Aarón Mayorga 2.6 h y Luis Martínez 2.6 h. Corte 14/07–04/08 (GitHub): Aarón 3.0 h; Luis Martínez 6.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1498,10 +1602,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I22" s="32" t="n">
-        <x:v>19</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="J22" s="32" t="n">
-        <x:v>19</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="K22" s="32" t="n">
         <x:v>0</x:v>
@@ -1516,10 +1620,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O22" s="32" t="n">
-        <x:v>38</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="P22" s="13" t="str">
-        <x:v>Pre-registro full-stack integrado en Administrativo: bandeja, creación, invitaciones, aceptación passwordless, auditoría e idempotencia. Pendientes clientes/tenants y aprovisionamiento Microsoft. Equipo del avance: Aarón Mayorga 19.0 h y Luis Martínez 19.0 h.</x:v>
+        <x:v>Pre-registro full-stack integrado en Administrativo: bandeja, creación, invitaciones, aceptación passwordless, auditoría e idempotencia. Pendientes clientes/tenants y aprovisionamiento Microsoft. Equipo del avance: Aarón Mayorga 19.0 h y Luis Martínez 19.0 h. Corte 14/07–04/08 (GitHub): Aarón 8.0 h; Luis Martínez 4.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1548,10 +1652,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I23" s="32" t="n">
-        <x:v>24.1</x:v>
+        <x:v>102.1</x:v>
       </x:c>
       <x:c r="J23" s="32" t="n">
-        <x:v>24.1</x:v>
+        <x:v>34.1</x:v>
       </x:c>
       <x:c r="K23" s="32" t="n">
         <x:v>0</x:v>
@@ -1566,10 +1670,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O23" s="32" t="n">
-        <x:v>48.2</x:v>
+        <x:v>136.2</x:v>
       </x:c>
       <x:c r="P23" s="13" t="str">
-        <x:v>Backend GTRS cerrado para 8 secciones, lectura, ETag y submit atómico; el frontend /formulario-gtrs-v2 aún usa definición y solicitud mock. Equipo del avance: Aarón Mayorga 24.1 h y Luis Martínez 24.1 h.</x:v>
+        <x:v>Backend GTRS cerrado para 8 secciones, lectura, ETag y submit atómico; el frontend /formulario-gtrs-v2 aún usa definición y solicitud mock. Equipo del avance: Aarón Mayorga 24.1 h y Luis Martínez 24.1 h. Corte 14/07–04/08 (GitHub): Aarón 8.0 h; Luis Martínez 10.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1598,10 +1702,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I24" s="32" t="n">
-        <x:v>16.6</x:v>
+        <x:v>21.6</x:v>
       </x:c>
       <x:c r="J24" s="32" t="n">
-        <x:v>16.6</x:v>
+        <x:v>19.6</x:v>
       </x:c>
       <x:c r="K24" s="32" t="n">
         <x:v>0</x:v>
@@ -1616,10 +1720,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O24" s="32" t="n">
-        <x:v>33.2</x:v>
+        <x:v>41.2</x:v>
       </x:c>
       <x:c r="P24" s="13" t="str">
-        <x:v>State machine, autorización y contratos de revisión presentes; integración funcional completa de revisión/UI pendiente. Equipo del avance: Aarón Mayorga 16.6 h y Luis Martínez 16.6 h.</x:v>
+        <x:v>State machine, autorización y contratos de revisión presentes; integración funcional completa de revisión/UI pendiente. Equipo del avance: Aarón Mayorga 16.6 h y Luis Martínez 16.6 h. Corte 14/07–04/08 (GitHub): Aarón 5.0 h; Luis Martínez 3.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1648,10 +1752,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I25" s="32" t="n">
-        <x:v>27.6</x:v>
+        <x:v>32.6</x:v>
       </x:c>
       <x:c r="J25" s="32" t="n">
-        <x:v>27.6</x:v>
+        <x:v>29.6</x:v>
       </x:c>
       <x:c r="K25" s="32" t="n">
         <x:v>0</x:v>
@@ -1666,10 +1770,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O25" s="32" t="n">
-        <x:v>55.2</x:v>
+        <x:v>62.2</x:v>
       </x:c>
       <x:c r="P25" s="13" t="str">
-        <x:v>Invitación, aceptación passwordless, Magic Link y acceso externo multiempresa implementados; captura GTRS vertical pendiente. Equipo del avance: Aarón Mayorga 27.6 h y Luis Martínez 27.6 h.</x:v>
+        <x:v>Invitación, aceptación passwordless, Magic Link y acceso externo multiempresa implementados; captura GTRS vertical pendiente. Equipo del avance: Aarón Mayorga 27.6 h y Luis Martínez 27.6 h. Corte 14/07–04/08 (GitHub): Aarón 5.0 h; Luis Martínez 2.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1698,10 +1802,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I26" s="32" t="n">
-        <x:v>7.8</x:v>
+        <x:v>11.8</x:v>
       </x:c>
       <x:c r="J26" s="32" t="n">
-        <x:v>7.8</x:v>
+        <x:v>8.8</x:v>
       </x:c>
       <x:c r="K26" s="32" t="n">
         <x:v>0</x:v>
@@ -1716,10 +1820,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O26" s="32" t="n">
-        <x:v>15.6</x:v>
+        <x:v>20.6</x:v>
       </x:c>
       <x:c r="P26" s="13" t="str">
-        <x:v>Pre-registro interno, guards, permisos y gestión de usuarios integrados; otros workspaces conservan mocks/prototipos. Equipo del avance: Aarón Mayorga 7.8 h y Luis Martínez 7.8 h.</x:v>
+        <x:v>Pre-registro interno, guards, permisos y gestión de usuarios integrados; otros workspaces conservan mocks/prototipos. Equipo del avance: Aarón Mayorga 7.8 h y Luis Martínez 7.8 h. Corte 14/07–04/08 (GitHub): Aarón 4.0 h; Luis Martínez 1.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1768,9 +1872,7 @@
       <x:c r="O27" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P27" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P27" s="13" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="n">
@@ -1818,9 +1920,7 @@
       <x:c r="O28" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P28" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P28" s="13" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="n">
@@ -1848,10 +1948,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I29" s="32" t="n">
-        <x:v>5.9</x:v>
+        <x:v>7.9</x:v>
       </x:c>
       <x:c r="J29" s="32" t="n">
-        <x:v>5.9</x:v>
+        <x:v>10.9</x:v>
       </x:c>
       <x:c r="K29" s="32" t="n">
         <x:v>0</x:v>
@@ -1866,10 +1966,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O29" s="32" t="n">
-        <x:v>11.8</x:v>
+        <x:v>18.8</x:v>
       </x:c>
       <x:c r="P29" s="13" t="str">
-        <x:v>Contexto canónico, handoffs, decisiones, autenticación, despliegue y runbooks actualizados al 10/08. Equipo del avance: Aarón Mayorga 5.9 h y Luis Martínez 5.9 h.</x:v>
+        <x:v>Contexto canónico, handoffs, decisiones, autenticación, despliegue y runbooks actualizados al 10/08. Equipo del avance: Aarón Mayorga 5.9 h y Luis Martínez 5.9 h. Corte 14/07–04/08 (GitHub): Aarón 2.0 h; Luis Martínez 5.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1898,10 +1998,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I30" s="32" t="n">
-        <x:v>4.5</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="J30" s="32" t="n">
-        <x:v>4.5</x:v>
+        <x:v>10.5</x:v>
       </x:c>
       <x:c r="K30" s="32" t="n">
         <x:v>0</x:v>
@@ -1916,10 +2016,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O30" s="32" t="n">
-        <x:v>9</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="P30" s="13" t="str">
-        <x:v>Cobertura automatizada amplia en frontend, API, Application, SQL y concurrencia; UAT aún no iniciado. Equipo del avance: Aarón Mayorga 4.5 h y Luis Martínez 4.5 h.</x:v>
+        <x:v>Cobertura automatizada amplia en frontend, API, Application, SQL y concurrencia; UAT aún no iniciado. Equipo del avance: Aarón Mayorga 4.5 h y Luis Martínez 4.5 h. Corte 14/07–04/08 (GitHub): Aarón 1.0 h; Luis Martínez 6.0 h.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1968,9 +2068,7 @@
       <x:c r="O31" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P31" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P31" s="13" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="n">
@@ -2018,9 +2116,7 @@
       <x:c r="O32" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P32" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P32" s="13" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="n">
@@ -2068,9 +2164,7 @@
       <x:c r="O33" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P33" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P33" s="13" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="n">
@@ -2218,9 +2312,7 @@
       <x:c r="O36" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P36" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P36" s="13" t="str"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="n">
@@ -2268,9 +2360,7 @@
       <x:c r="O37" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P37" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P37" s="13" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="n">
@@ -2318,9 +2408,7 @@
       <x:c r="O38" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P38" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P38" s="13" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="n">
@@ -2368,9 +2456,7 @@
       <x:c r="O39" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P39" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P39" s="13" t="str"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="n">
@@ -2418,9 +2504,7 @@
       <x:c r="O40" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P40" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P40" s="13" t="str"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="n">
@@ -2468,9 +2552,7 @@
       <x:c r="O41" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P41" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P41" s="13" t="str"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="n">
@@ -2518,9 +2600,7 @@
       <x:c r="O42" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P42" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P42" s="13" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" t="n">
@@ -2568,9 +2648,7 @@
       <x:c r="O43" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P43" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P43" s="13" t="str"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" t="n">
@@ -2618,9 +2696,7 @@
       <x:c r="O44" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P44" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P44" s="13" t="str"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="n">
@@ -2668,9 +2744,7 @@
       <x:c r="O45" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P45" s="13" t="str">
-        <x:v> </x:v>
-      </x:c>
+      <x:c r="P45" s="13" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2742,7 +2816,7 @@
         <x:v>109</x:v>
       </x:c>
       <x:c r="E3" s="32" t="n">
-        <x:v>41.6</x:v>
+        <x:v>156.6</x:v>
       </x:c>
       <x:c r="F3" s="32" t="n">
         <x:v>92.8</x:v>
@@ -2762,7 +2836,7 @@
         <x:v>781</x:v>
       </x:c>
       <x:c r="E4" s="32" t="n">
-        <x:v>227.4</x:v>
+        <x:v>400.4</x:v>
       </x:c>
       <x:c r="F4" s="32" t="n">
         <x:v>49.1</x:v>
@@ -2782,7 +2856,7 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="E5" s="32" t="n">
-        <x:v>9</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F5" s="32" t="n">
         <x:v>17.8</x:v>
@@ -2891,7 +2965,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E3" s="32" t="n">
-        <x:v>182</x:v>
+        <x:v>335</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2908,7 +2982,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="E4" s="32" t="n">
-        <x:v>146</x:v>
+        <x:v>238</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2925,7 +2999,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E5" s="32" t="n">
-        <x:v>12</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2998,7 +3072,7 @@
     <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="70" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="72" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -3036,7 +3110,7 @@
         <x:v>Notas / evidencia</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="50" customHeight="1">
+    <x:row r="2" ht="105" customHeight="1">
       <x:c r="A2" s="9" t="n">
         <x:v>46238</x:v>
       </x:c>
@@ -3062,16 +3136,16 @@
         <x:v>0.023</x:v>
       </x:c>
       <x:c r="I2" s="11" t="str">
-        <x:v>feature/backend-capabilities</x:v>
+        <x:v>main</x:v>
       </x:c>
       <x:c r="J2" s="11" t="str">
-        <x:v>b26f13f</x:v>
+        <x:v>31ecaf5..95a1b5b</x:v>
       </x:c>
       <x:c r="K2" s="12" t="str">
-        <x:v>Primer corte validado contra código ejecutable, migraciones, endpoints, pruebas y configuración funcional. Medición operativa ponderada por horas planificadas.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="110" customHeight="1">
+        <x:v>Corte 14/07–04/08 validado contra GitHub: 364 commits (355 sin merge + 9 merges), 443 archivos modificados y 16 días-persona activos. Estimación conservadora de 128.0 h omitidas: Aarón 56.0 h y Luis Martínez 72.0 h, a 8 h por día activo y distribuidas por entregable. Evidencia: https://github.com/Grant-Thornton-Costa-Rica/FARO/compare/31ecaf5...95a1b5b</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="125" customHeight="1">
       <x:c r="A3" s="27" t="n">
         <x:v>46247.75</x:v>
       </x:c>
@@ -3103,13 +3177,345 @@
         <x:v>fdbea06</x:v>
       </x:c>
       <x:c r="K3" s="31" t="str">
-        <x:v>Corte validado sobre FARO main@fdbea06. Pre-registro full-stack integrado dentro de Administrativo: creación, bandeja, invitación/reenvío/revocación, aceptación passwordless, auditoría, idempotencia y alcance global Riesgo/Admin. También se reconoce el cierre backend GTRS de 8 secciones con ETag y gate de completitud. Pendientes principales: integración vertical del frontend GTRS, aprovisionamiento Microsoft/Entra y UAT. Horas del avance redistribuidas: 260.0 h totales, 130.0 h Aarón Mayorga y 130.0 h Luis Martínez; sin participación de Daniel Pulido, Luis Montero, Karol ni Jorge Jiménez en las tareas que avanzaron.</x:v>
+        <x:v>Corte validado sobre FARO main@fdbea06. Pre-registro full-stack integrado dentro de Administrativo: creación, bandeja, invitación/reenvío/revocación, aceptación passwordless, auditoría, idempotencia y alcance global Riesgo/Admin. También se reconoce el cierre backend GTRS de 8 secciones con ETag y gate de completitud. Pendientes principales: integración vertical del frontend GTRS, aprovisionamiento Microsoft/Entra y UAT. Horas del avance redistribuidas: 260.0 h totales, 130.0 h Aarón Mayorga y 130.0 h Luis Martínez; sin participación de Daniel Pulido, Luis Montero, Karol ni Jorge Jiménez en las tareas que avanzaron. Acumulado al 13/08: 655.0 h = 267.0 h de línea base al 13/07 + 128.0 h estimadas del corte 04/08 + 260.0 h del corte 13/08.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0f84c146ade4c8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99108d52c6e8453f"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="8" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="35" t="str">
+        <x:v>Estimación de horas omitidas · Corte 14/07–04/08/2026</x:v>
+      </x:c>
+      <x:c r="B1" s="35"/>
+      <x:c r="C1" s="35"/>
+      <x:c r="D1" s="35"/>
+      <x:c r="E1" s="35"/>
+      <x:c r="F1" s="35"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="5"/>
+      <x:c r="B2" s="5"/>
+      <x:c r="C2" s="5"/>
+      <x:c r="D2" s="5"/>
+      <x:c r="E2" s="5"/>
+      <x:c r="F2" s="5"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="51" t="str">
+        <x:v>Rango Git</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>31ecaf5..95a1b5b</x:v>
+      </x:c>
+      <x:c r="C3" s="5"/>
+      <x:c r="D3" s="5"/>
+      <x:c r="E3" s="5"/>
+      <x:c r="F3" s="5"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="51" t="str">
+        <x:v>Fuente GitHub</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>https://github.com/Grant-Thornton-Costa-Rica/FARO/compare/31ecaf5...95a1b5b</x:v>
+      </x:c>
+      <x:c r="C4" s="5"/>
+      <x:c r="D4" s="5"/>
+      <x:c r="E4" s="5"/>
+      <x:c r="F4" s="5"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="51" t="str">
+        <x:v>Commits totales</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="n">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="C5" s="5"/>
+      <x:c r="D5" s="5"/>
+      <x:c r="E5" s="5"/>
+      <x:c r="F5" s="5"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="51" t="str">
+        <x:v>Commits sin merge</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="n">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="C6" s="5"/>
+      <x:c r="D6" s="5"/>
+      <x:c r="E6" s="5"/>
+      <x:c r="F6" s="5"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="51" t="str">
+        <x:v>Merges</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C7" s="5"/>
+      <x:c r="D7" s="5"/>
+      <x:c r="E7" s="5"/>
+      <x:c r="F7" s="5"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="51" t="str">
+        <x:v>Archivos modificados</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="n">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="C8" s="5"/>
+      <x:c r="D8" s="5"/>
+      <x:c r="E8" s="5"/>
+      <x:c r="F8" s="5"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="51" t="str">
+        <x:v>Inserciones / eliminaciones</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>84,623 / 5,354</x:v>
+      </x:c>
+      <x:c r="C9" s="5"/>
+      <x:c r="D9" s="5"/>
+      <x:c r="E9" s="5"/>
+      <x:c r="F9" s="5"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="51" t="str">
+        <x:v>Método</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="str">
+        <x:v>8 horas por día-persona activo; contraste con entregables y cambios del repositorio.</x:v>
+      </x:c>
+      <x:c r="C10" s="5"/>
+      <x:c r="D10" s="5"/>
+      <x:c r="E10" s="5"/>
+      <x:c r="F10" s="5"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="5"/>
+      <x:c r="B11" s="5"/>
+      <x:c r="C11" s="5"/>
+      <x:c r="D11" s="5"/>
+      <x:c r="E11" s="5"/>
+      <x:c r="F11" s="5"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="35" t="str">
+        <x:v>Persona</x:v>
+      </x:c>
+      <x:c r="B12" s="35" t="str">
+        <x:v>Commits</x:v>
+      </x:c>
+      <x:c r="C12" s="35" t="str">
+        <x:v>Días activos</x:v>
+      </x:c>
+      <x:c r="D12" s="35" t="str">
+        <x:v>Horas/día</x:v>
+      </x:c>
+      <x:c r="E12" s="35" t="str">
+        <x:v>Horas estimadas</x:v>
+      </x:c>
+      <x:c r="F12" s="5"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="5" t="str">
+        <x:v>Aarón Mayorga</x:v>
+      </x:c>
+      <x:c r="B13" s="52" t="n">
+        <x:v>263</x:v>
+      </x:c>
+      <x:c r="C13" s="52" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D13" s="52" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E13" s="52" t="n">
+        <x:f>C13*D13</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="F13" s="5"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="5" t="str">
+        <x:v>Luis Martínez</x:v>
+      </x:c>
+      <x:c r="B14" s="52" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="C14" s="52" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D14" s="52" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E14" s="52" t="n">
+        <x:f>C14*D14</x:f>
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="F14" s="5"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="53" t="str">
+        <x:v>Total</x:v>
+      </x:c>
+      <x:c r="B15" s="54" t="n">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="C15" s="54" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D15" s="54"/>
+      <x:c r="E15" s="54" t="n">
+        <x:f>SUM(E13:E14)</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F15" s="5"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="5"/>
+      <x:c r="B16" s="5"/>
+      <x:c r="C16" s="5"/>
+      <x:c r="D16" s="5"/>
+      <x:c r="E16" s="5"/>
+      <x:c r="F16" s="5"/>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="45" t="str">
+        <x:v>Criterio: los commits prueban actividad y alcance, pero no se convierten individualmente en horas. La estimación usa días-persona activos y se distribuye entre tareas con entregables verificables. No se atribuyeron horas del intervalo a personas sin commits.</x:v>
+      </x:c>
+      <x:c r="B17" s="45"/>
+      <x:c r="C17" s="45"/>
+      <x:c r="D17" s="45"/>
+      <x:c r="E17" s="45"/>
+      <x:c r="F17" s="45"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="5"/>
+      <x:c r="B18" s="5"/>
+      <x:c r="C18" s="5"/>
+      <x:c r="D18" s="5"/>
+      <x:c r="E18" s="5"/>
+      <x:c r="F18" s="5"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="55" t="str">
+        <x:v>Componente acumulado</x:v>
+      </x:c>
+      <x:c r="B19" s="55" t="str">
+        <x:v>Aarón</x:v>
+      </x:c>
+      <x:c r="C19" s="55" t="str">
+        <x:v>Luis Martínez</x:v>
+      </x:c>
+      <x:c r="D19" s="55" t="str">
+        <x:v>Otros históricos</x:v>
+      </x:c>
+      <x:c r="E19" s="55" t="str">
+        <x:v>Total</x:v>
+      </x:c>
+      <x:c r="F19" s="5"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="5" t="str">
+        <x:v>Línea base al 13/07</x:v>
+      </x:c>
+      <x:c r="B20" s="52" t="n">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="C20" s="52" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D20" s="52" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="E20" s="52" t="n">
+        <x:v>267</x:v>
+      </x:c>
+      <x:c r="F20" s="5"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="5" t="str">
+        <x:v>Horas omitidas del corte 04/08</x:v>
+      </x:c>
+      <x:c r="B21" s="52" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C21" s="52" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="D21" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="52" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F21" s="5"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="5" t="str">
+        <x:v>Horas del corte 13/08</x:v>
+      </x:c>
+      <x:c r="B22" s="52" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="C22" s="52" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="D22" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="52" t="n">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="F22" s="5"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="56" t="str">
+        <x:v>Acumulado</x:v>
+      </x:c>
+      <x:c r="B23" s="57" t="n">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="C23" s="57" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="D23" s="57" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="E23" s="57" t="n">
+        <x:v>655</x:v>
+      </x:c>
+      <x:c r="F23" s="5"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A17:F17"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>